<commit_message>
Add import-advisor.bat + IMPORT_ONLY filter for per-advisor imports
- import-advisor.bat: prompts for advisor name + sections, runs a dry-run,
  then the real import from FA_Data\<name>\ (Windows double-click workflow)
- import-from-excel: IMPORT_ONLY env limits which sections run (clients/
  portfolio/insurance/assets)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FA_Data/TAN TIAN YING/1_Clients_Database.xlsx
+++ b/FA_Data/TAN TIAN YING/1_Clients_Database.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{54059AD8-0B44-4479-ABF1-4B2BA8B5980B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" firstSheet="1" activeTab="1"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="📋 READ ME FIRST" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Clients Data Entry" state="visible" r:id="rId5"/>
+    <sheet name="📋 READ ME FIRST" sheetId="1" r:id="rId1"/>
+    <sheet name="Clients Data Entry" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="53">
   <si>
     <t/>
   </si>
@@ -156,106 +157,124 @@
   </si>
   <si>
     <t>e.g. client@email.com</t>
+  </si>
+  <si>
+    <t>TEO GUO CHAN</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Moderate</t>
+  </si>
+  <si>
+    <t>HNW</t>
+  </si>
+  <si>
+    <t>lovelytian97@gmail.com</t>
+  </si>
+  <si>
+    <t>CASH FLOW, RETIREMENT, EDUCATION PLANNING,</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="14" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="16"/>
       <color rgb="FF0A4A14"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="16"/>
-      <name val="Arial"/>
     </font>
     <font>
       <i/>
+      <sz val="11"/>
       <color rgb="FF4A7A4E"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FF0F2012"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF1A1A1A"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF2D6A35"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF1565C0"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FFC62828"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="14"/>
       <color rgb="FFE8F5EA"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFA8D5AC"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFE8F5EA"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
       <i/>
+      <sz val="9"/>
       <color rgb="FF555555"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="9"/>
-      <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="10">
@@ -345,10 +364,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -383,29 +403,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -742,16 +766,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:C25"/>
-  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -762,7 +786,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -773,7 +797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" ht="11.1" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="11.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -784,7 +808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -795,7 +819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -806,7 +830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -817,7 +841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -828,7 +852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -839,7 +863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -850,7 +874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -861,7 +885,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="11.1" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="11.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -872,7 +896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -883,7 +907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -894,7 +918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -905,7 +929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -916,7 +940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -927,7 +951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="11.1" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="11.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -938,7 +962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>0</v>
       </c>
@@ -949,7 +973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -960,7 +984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -971,7 +995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="10.15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="10.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>0</v>
       </c>
@@ -984,14 +1008,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M54"/>
-  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.7109375" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:M53"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="36" style="10" customWidth="1"/>
     <col min="2" max="2" width="14" style="10" customWidth="1"/>
@@ -1004,473 +1028,291 @@
     <col min="11" max="11" width="44" style="10" customWidth="1"/>
     <col min="12" max="12" width="20" style="11" customWidth="1"/>
     <col min="13" max="13" width="30" style="10" customWidth="1"/>
-    <col min="14" max="16384" width="8.7109375" style="10" customWidth="1"/>
+    <col min="14" max="14" width="8.7265625" style="10" customWidth="1"/>
+    <col min="15" max="16384" width="8.7265625" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:13" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-    </row>
-    <row r="2" ht="20.1" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+    </row>
+    <row r="2" spans="1:13" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-    </row>
-    <row r="3" ht="32.1" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="18"/>
+    </row>
+    <row r="3" spans="1:13" ht="32.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="G3" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="H3" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="I3" s="14" t="s">
+      <c r="I3" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="J3" s="14" t="s">
+      <c r="J3" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="K3" s="14" t="s">
+      <c r="K3" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="14" t="s">
+      <c r="L3" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="M3" s="14" t="s">
+      <c r="M3" s="12" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="4" ht="28.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+    <row r="4" spans="1:13" ht="28.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="I4" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="J4" s="15" t="s">
+      <c r="J4" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="K4" s="15" t="s">
+      <c r="K4" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="L4" s="15" t="s">
+      <c r="L4" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="M4" s="15" t="s">
+      <c r="M4" s="13" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="5" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="10"/>
-    </row>
-    <row r="6" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="10"/>
-    </row>
-    <row r="7" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="10"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="10"/>
-    </row>
-    <row r="8" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="10"/>
-    </row>
-    <row r="9" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="10"/>
-    </row>
-    <row r="10" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="10"/>
-    </row>
-    <row r="11" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="10"/>
-    </row>
-    <row r="12" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="10"/>
-    </row>
-    <row r="13" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="10"/>
-    </row>
-    <row r="14" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="17"/>
-    </row>
-    <row r="15" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="17"/>
-    </row>
-    <row r="16" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="17"/>
-    </row>
-    <row r="17" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="17"/>
-    </row>
-    <row r="18" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="17"/>
-    </row>
-    <row r="19" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="11"/>
-      <c r="M19" s="17"/>
-    </row>
-    <row r="20" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" s="10"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="16"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="17"/>
-    </row>
-    <row r="21" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="10"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
+    <row r="5" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="10">
+        <v>2000000</v>
+      </c>
+      <c r="F5" s="10">
+        <v>10000</v>
+      </c>
+      <c r="G5" s="14">
+        <v>34434</v>
+      </c>
+      <c r="H5" s="14"/>
+      <c r="K5" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="L5" s="11">
+        <v>1139433194</v>
+      </c>
+      <c r="M5" s="19" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+    </row>
+    <row r="8" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+    </row>
+    <row r="9" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+    </row>
+    <row r="10" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+    </row>
+    <row r="11" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+    </row>
+    <row r="12" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
+    </row>
+    <row r="13" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="M13" s="15"/>
+    </row>
+    <row r="14" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+      <c r="M14" s="15"/>
+    </row>
+    <row r="15" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="M15" s="15"/>
+    </row>
+    <row r="16" spans="1:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="M16" s="15"/>
+    </row>
+    <row r="17" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="M17" s="15"/>
+    </row>
+    <row r="18" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="M18" s="15"/>
+    </row>
+    <row r="19" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="M19" s="15"/>
+    </row>
+    <row r="20" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="M20" s="15"/>
+    </row>
+    <row r="21" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="17"/>
-    </row>
-    <row r="22" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="17"/>
-    </row>
-    <row r="23" ht="22.15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-    </row>
-    <row r="24" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" ht="22.15" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="M21" s="15"/>
+    </row>
+    <row r="22" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G22" s="16"/>
+      <c r="H22" s="16"/>
+      <c r="M22" s="11"/>
+    </row>
+    <row r="23" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="24" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="25" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="26" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="27" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="28" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="29" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="30" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="31" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="32" spans="7:13" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="33" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="34" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="35" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="36" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="37" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="38" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="39" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="40" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="41" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="42" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="43" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="44" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="45" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="46" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="47" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="48" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="49" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="50" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="51" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="52" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="53" ht="22.15" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A2:M2"/>
   </mergeCells>
-  <dataValidations count="8">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid option" error="Please choose: Active | Prospect | Inactive" sqref="B10:B54">
+  <dataValidations count="4">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Active | Prospect | Inactive" sqref="B5:B53" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Active,Prospect,Inactive"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid option" error="Please choose: Active | Prospect | Inactive" sqref="B5:B54">
-      <formula1>"Active,Prospect,Inactive"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid option" error="Please choose: Affluent | Mass Affluent | HNW | UHNW" sqref="C10:C54">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Affluent | Mass Affluent | HNW | UHNW" sqref="C5:C53" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"Affluent,Mass Affluent,HNW,UHNW"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid option" error="Please choose: Affluent | Mass Affluent | HNW | UHNW" sqref="C5:C54">
-      <formula1>"Affluent,Mass Affluent,HNW,UHNW"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid option" error="Please choose: Conservative | Moderate | Aggressive" sqref="D10:D54">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Conservative | Moderate | Aggressive" sqref="D5:D53" xr:uid="{00000000-0002-0000-0100-000004000000}">
       <formula1>"Conservative,Moderate,Aggressive"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid option" error="Please choose: Conservative | Moderate | Aggressive" sqref="D5:D54">
-      <formula1>"Conservative,Moderate,Aggressive"</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Date format" prompt="Enter date as YYYY-MM-DD  e.g. 2026-05-19" sqref="G10:J54">
-      <formula1>TRUE</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Date format" prompt="Enter date as YYYY-MM-DD  e.g. 2026-05-19" sqref="G5:J54">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Date format" prompt="Enter date as YYYY-MM-DD  e.g. 2026-05-19" sqref="G5:J53" xr:uid="{00000000-0002-0000-0100-000006000000}">
       <formula1>TRUE</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="M5" r:id="rId1" xr:uid="{A1F92E3E-18AC-4769-9125-F391B854D2F6}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>